<commit_message>
Bom update and cleanup
</commit_message>
<xml_diff>
--- a/main_hw/SUMEC_MK_V/bom/SUMEC_MK_V.xlsx
+++ b/main_hw/SUMEC_MK_V/bom/SUMEC_MK_V.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MenMe\GitHub\Sumec-MiniSumo-HW\main_hw\SUMEC_MK_V\bom\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MenMe\Documents\GitHub\Sumec-MiniSumo-HW\main_hw\SUMEC_MK_V\bom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F8EF6A6-0E47-455C-A723-6B0CBACD71D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FE802D3-71E3-4C55-9E7D-7F90F82FDEF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{318D0819-0F8D-4535-926A-50240C04F6C9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{318D0819-0F8D-4535-926A-50240C04F6C9}"/>
   </bookViews>
   <sheets>
     <sheet name="SUMEC_MK_V" sheetId="1" r:id="rId1"/>
@@ -1459,18 +1459,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C378E24-255E-4758-9EA3-ADC3BD7350B6}">
   <dimension ref="A1:F45"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="37.81640625" style="9" customWidth="1"/>
-    <col min="2" max="2" width="24.90625" style="9" customWidth="1"/>
-    <col min="3" max="3" width="13.1796875" style="9" customWidth="1"/>
+    <col min="1" max="1" width="37.77734375" style="9" customWidth="1"/>
+    <col min="2" max="2" width="24.88671875" style="9" customWidth="1"/>
+    <col min="3" max="3" width="13.21875" style="9" customWidth="1"/>
     <col min="4" max="4" width="36" style="9" customWidth="1"/>
     <col min="5" max="5" width="35" style="9" customWidth="1"/>
-    <col min="6" max="6" width="26.81640625" style="9" customWidth="1"/>
-    <col min="7" max="16384" width="8.7265625" style="9"/>
+    <col min="6" max="6" width="26.77734375" style="9" customWidth="1"/>
+    <col min="7" max="16384" width="8.77734375" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>97</v>
       </c>
@@ -1490,7 +1490,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>2</v>
       </c>
@@ -1510,7 +1510,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="9" t="s">
         <v>4</v>
       </c>
@@ -1530,7 +1530,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>7</v>
       </c>
@@ -1550,7 +1550,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="9" t="s">
         <v>10</v>
       </c>
@@ -1570,7 +1570,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>13</v>
       </c>
@@ -1590,7 +1590,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
         <v>15</v>
       </c>
@@ -1610,7 +1610,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
         <v>18</v>
       </c>
@@ -1630,7 +1630,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="E9" s="6" t="s">
         <v>130</v>
       </c>
@@ -1638,7 +1638,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="E10" s="6" t="s">
         <v>131</v>
       </c>
@@ -1646,7 +1646,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
         <v>21</v>
       </c>
@@ -1666,7 +1666,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
         <v>24</v>
       </c>
@@ -1686,7 +1686,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="9" t="s">
         <v>27</v>
       </c>
@@ -1706,7 +1706,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="9" t="s">
         <v>29</v>
       </c>
@@ -1726,7 +1726,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="9" t="s">
         <v>32</v>
       </c>
@@ -1746,7 +1746,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="9" t="s">
         <v>35</v>
       </c>
@@ -1766,7 +1766,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="9" t="s">
         <v>38</v>
       </c>
@@ -1786,7 +1786,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="9" t="s">
         <v>41</v>
       </c>
@@ -1806,7 +1806,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="9" t="s">
         <v>44</v>
       </c>
@@ -1826,7 +1826,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="9" t="s">
         <v>47</v>
       </c>
@@ -1846,7 +1846,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="9" t="s">
         <v>50</v>
       </c>
@@ -1866,7 +1866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="9" t="s">
         <v>53</v>
       </c>
@@ -1886,7 +1886,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="9" t="s">
         <v>56</v>
       </c>
@@ -1906,7 +1906,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="9" t="s">
         <v>58</v>
       </c>
@@ -1926,7 +1926,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="9" t="s">
         <v>60</v>
       </c>
@@ -1946,7 +1946,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="9" t="s">
         <v>62</v>
       </c>
@@ -1966,7 +1966,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="9" t="s">
         <v>64</v>
       </c>
@@ -1986,7 +1986,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="9" t="s">
         <v>66</v>
       </c>
@@ -2006,7 +2006,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="9" t="s">
         <v>68</v>
       </c>
@@ -2026,7 +2026,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="9" t="s">
         <v>70</v>
       </c>
@@ -2046,7 +2046,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="9" t="s">
         <v>72</v>
       </c>
@@ -2066,7 +2066,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="9" t="s">
         <v>134</v>
       </c>
@@ -2086,7 +2086,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="9" t="s">
         <v>75</v>
       </c>
@@ -2106,7 +2106,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="9" t="s">
         <v>77</v>
       </c>
@@ -2126,7 +2126,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="9" t="s">
         <v>79</v>
       </c>
@@ -2146,7 +2146,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="9" t="s">
         <v>81</v>
       </c>
@@ -2166,7 +2166,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="9" t="s">
         <v>84</v>
       </c>
@@ -2186,7 +2186,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="9" t="s">
         <v>86</v>
       </c>
@@ -2206,7 +2206,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="9" t="s">
         <v>89</v>
       </c>
@@ -2226,7 +2226,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="9" t="s">
         <v>92</v>
       </c>
@@ -2246,7 +2246,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="9" t="s">
         <v>95</v>
       </c>
@@ -2263,7 +2263,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C43" s="9">
         <v>1</v>
       </c>
@@ -2274,7 +2274,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="9" t="s">
         <v>149</v>
       </c>
@@ -2288,7 +2288,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="C45" s="9">
         <v>1</v>
       </c>

</xml_diff>